<commit_message>
Added Request Body to test POST calls
Added Request Body to test POST calls
</commit_message>
<xml_diff>
--- a/Issues.xlsx
+++ b/Issues.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/padmaramaraju/Work/2026-2027/Claude/Projects/CoWork/Lohitas/lohitas-middleware/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/padmaramaraju/Work/2026-2027/Claude/Projects/CoWork/Lohitas/naimix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{100E3B4F-45F0-DF47-9056-1F20F5D22099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{70633AAF-CD21-EB4F-A0F0-6942A9091777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5040" yWindow="1540" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{C090ABE5-14E0-B34C-911F-B2115D1F2353}"/>
+    <workbookView xWindow="5040" yWindow="1540" windowWidth="27640" windowHeight="16940" activeTab="1" xr2:uid="{C090ABE5-14E0-B34C-911F-B2115D1F2353}"/>
   </bookViews>
   <sheets>
     <sheet name="Issues" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>Backend URL must be mandatory for connection</t>
   </si>
@@ -148,6 +148,9 @@
   </si>
   <si>
     <t>Vibe coding enabled with industry standrd tools like Claude and Cursor using the MCP tool</t>
+  </si>
+  <si>
+    <t>Documentation Web Site and jump to documentation from any screen</t>
   </si>
 </sst>
 </file>
@@ -577,7 +580,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17CEC5DA-1334-C244-ACE2-BED76F7DED99}">
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="52.83203125" customWidth="1"/>
@@ -660,51 +663,56 @@
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" s="3" t="s">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" s="3" t="s">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
         <v>25</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
         <v>28</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Swagger and MCP Downloads for a workspace
Added Swagger Download for a workspace.  Now users can download Swagger for the workspace.  It covers all the end points and auth providers defined in the workspace at the time if download.

Added MCP Download for a workspace.  Now users can download MCP server for the workspace.  It covers all the end points and auth providers defined in the workspace at the time if download.  The MCP server can be configured in any MCP client (like Claude) and the end points can be invoked with natural language.
</commit_message>
<xml_diff>
--- a/Issues.xlsx
+++ b/Issues.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/padmaramaraju/Work/2026-2027/Claude/Projects/CoWork/Lohitas/naimix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{70633AAF-CD21-EB4F-A0F0-6942A9091777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4498BE33-6E16-4A47-87F1-6E20C6B7818D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5040" yWindow="1540" windowWidth="27640" windowHeight="16940" activeTab="1" xr2:uid="{C090ABE5-14E0-B34C-911F-B2115D1F2353}"/>
   </bookViews>
@@ -19,7 +19,6 @@
     <sheet name="Foundry vs Lohitas Middleware" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>Backend URL must be mandatory for connection</t>
   </si>
@@ -151,13 +150,42 @@
   </si>
   <si>
     <t>Documentation Web Site and jump to documentation from any screen</t>
+  </si>
+  <si>
+    <r>
+      <t>"message"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Monaco"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF0451A5"/>
+        <rFont val="Monaco"/>
+        <family val="2"/>
+      </rPr>
+      <t>"This endpoint requires authentication. Log in via POST /auth/login/duende-oauth2-cc and send the returned token as \"Authorization: Bearer &lt;token&gt;\"."</t>
+    </r>
+  </si>
+  <si>
+    <t>Generate MCP for a BFF</t>
+  </si>
+  <si>
+    <t>Configure BFF by linking and grouping end points</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -176,6 +204,24 @@
       <sz val="14"/>
       <color rgb="FF565959"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Monaco"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFA31515"/>
+      <name val="Monaco"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0451A5"/>
+      <name val="Monaco"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -199,7 +245,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -210,6 +256,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -580,7 +627,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17CEC5DA-1334-C244-ACE2-BED76F7DED99}">
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="52.83203125" customWidth="1"/>
@@ -621,99 +668,117 @@
         <v>9</v>
       </c>
     </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" s="2"/>
+    </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
-        <v>16</v>
+      <c r="A16" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>19</v>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A28" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A29" s="3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
+    <row r="35" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="3" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" s="6" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>